<commit_message>
fix: separate blank template from example archive
</commit_message>
<xml_diff>
--- a/skill/travel-os/assets/TravelOS-Template.xlsx
+++ b/skill/travel-os/assets/TravelOS-Template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travel Overview" sheetId="1" r:id="R1923f46351a44bca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Plan" sheetId="2" r:id="R57f2af995ad545fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="3" r:id="R3f382a0ca7ce463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="4" r:id="Re882fef17dff4f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferences" sheetId="5" r:id="R10c94c6a9c9a44f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="6" r:id="R0d82132e5d19404c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" r:id="R5b4c9e3a47264ad5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposals" sheetId="8" r:id="R0f4a7277c3624dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travel Overview" sheetId="1" r:id="Rb064bddc82b44833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Plan" sheetId="2" r:id="R90206dae9334462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="3" r:id="Rc155e68ab1c24824"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="4" r:id="R598f5d44f3ad4f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferences" sheetId="5" r:id="R4681bcd0bed946a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="6" r:id="Rdba29f382d9d4841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" r:id="Rc3b476cd2b3e4bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposals" sheetId="8" r:id="R974b8a2f51674eca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -281,6 +281,157 @@
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TravelOverview" displayName="TravelOverview" ref="A2:L4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="Trip ID"/>
+    <x:tableColumn id="2" name="旅行标题"/>
+    <x:tableColumn id="3" name="目的地"/>
+    <x:tableColumn id="4" name="开始日期"/>
+    <x:tableColumn id="5" name="结束日期"/>
+    <x:tableColumn id="6" name="人数"/>
+    <x:tableColumn id="7" name="负责人"/>
+    <x:tableColumn id="8" name="Active Version"/>
+    <x:tableColumn id="9" name="旅行阶段"/>
+    <x:tableColumn id="10" name="状态"/>
+    <x:tableColumn id="11" name="主时区"/>
+    <x:tableColumn id="12" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DailyPlan" displayName="DailyPlan" ref="A2:Q5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="17">
+    <x:tableColumn id="1" name="项目ID"/>
+    <x:tableColumn id="2" name="版本"/>
+    <x:tableColumn id="3" name="日期"/>
+    <x:tableColumn id="4" name="开始"/>
+    <x:tableColumn id="5" name="结束"/>
+    <x:tableColumn id="6" name="时区"/>
+    <x:tableColumn id="7" name="城市"/>
+    <x:tableColumn id="8" name="活动"/>
+    <x:tableColumn id="9" name="地点"/>
+    <x:tableColumn id="10" name="交通"/>
+    <x:tableColumn id="11" name="预订ID"/>
+    <x:tableColumn id="12" name="执行状态"/>
+    <x:tableColumn id="13" name="费用"/>
+    <x:tableColumn id="14" name="币种"/>
+    <x:tableColumn id="15" name="来源"/>
+    <x:tableColumn id="16" name="核验时间"/>
+    <x:tableColumn id="17" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Bookings" displayName="Bookings" ref="A2:N4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="14">
+    <x:tableColumn id="1" name="预订ID"/>
+    <x:tableColumn id="2" name="类别"/>
+    <x:tableColumn id="3" name="供应方"/>
+    <x:tableColumn id="4" name="开始时间"/>
+    <x:tableColumn id="5" name="结束时间"/>
+    <x:tableColumn id="6" name="城市"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="可退"/>
+    <x:tableColumn id="9" name="金额"/>
+    <x:tableColumn id="10" name="币种"/>
+    <x:tableColumn id="11" name="凭证位置"/>
+    <x:tableColumn id="12" name="来源"/>
+    <x:tableColumn id="13" name="核验时间"/>
+    <x:tableColumn id="14" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Checklist" displayName="Checklist" ref="A2:I4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务ID"/>
+    <x:tableColumn id="2" name="类别"/>
+    <x:tableColumn id="3" name="任务"/>
+    <x:tableColumn id="4" name="负责人"/>
+    <x:tableColumn id="5" name="截止日期"/>
+    <x:tableColumn id="6" name="状态"/>
+    <x:tableColumn id="7" name="依赖"/>
+    <x:tableColumn id="8" name="关联ID"/>
+    <x:tableColumn id="9" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Preferences" displayName="Preferences" ref="A2:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="偏好ID"/>
+    <x:tableColumn id="2" name="范围"/>
+    <x:tableColumn id="3" name="类别"/>
+    <x:tableColumn id="4" name="优先级"/>
+    <x:tableColumn id="5" name="适用人"/>
+    <x:tableColumn id="6" name="偏好或约束"/>
+    <x:tableColumn id="7" name="证据"/>
+    <x:tableColumn id="8" name="置信度"/>
+    <x:tableColumn id="9" name="生效日期"/>
+    <x:tableColumn id="10" name="失效日期"/>
+    <x:tableColumn id="11" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ChangeLog" displayName="ChangeLog" ref="A2:G4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="版本"/>
+    <x:tableColumn id="2" name="创建时间"/>
+    <x:tableColumn id="3" name="作者"/>
+    <x:tableColumn id="4" name="原因"/>
+    <x:tableColumn id="5" name="变更摘要"/>
+    <x:tableColumn id="6" name="上一版本"/>
+    <x:tableColumn id="7" name="档案哈希"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Members" displayName="Members" ref="A2:G5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="成员ID"/>
+    <x:tableColumn id="2" name="显示名"/>
+    <x:tableColumn id="3" name="角色"/>
+    <x:tableColumn id="4" name="同行关系"/>
+    <x:tableColumn id="5" name="本次需求"/>
+    <x:tableColumn id="6" name="权限"/>
+    <x:tableColumn id="7" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Proposals" displayName="Proposals" ref="A2:J4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="提案ID"/>
+    <x:tableColumn id="2" name="提交人"/>
+    <x:tableColumn id="3" name="日期"/>
+    <x:tableColumn id="4" name="影响项目或日期"/>
+    <x:tableColumn id="5" name="提案"/>
+    <x:tableColumn id="6" name="原因"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="决策人"/>
+    <x:tableColumn id="9" name="处理结果"/>
+    <x:tableColumn id="10" name="结果版本"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -536,56 +687,32 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>DEMO-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>示例城市周末</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="D3" s="17" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E3" s="17" t="d">
-        <x:v>2030-05-03T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="H3" s="21" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="I3" s="12" t="str">
-        <x:v>行前规划</x:v>
-      </x:c>
-      <x:c r="J3" s="12" t="str">
-        <x:v>Active</x:v>
-      </x:c>
-      <x:c r="K3" s="12" t="str">
-        <x:v>Asia/Shanghai</x:v>
-      </x:c>
-      <x:c r="L3" s="13" t="str">
-        <x:v>本行仅为虚构示例，请替换</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="12"/>
+      <x:c r="G3" s="12"/>
+      <x:c r="H3" s="21"/>
+      <x:c r="I3" s="12"/>
+      <x:c r="J3" s="12"/>
+      <x:c r="K3" s="12"/>
+      <x:c r="L3" s="13"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="15" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="15"/>
       <x:c r="D4" s="18"/>
       <x:c r="E4" s="18"/>
       <x:c r="F4" s="15"/>
-      <x:c r="G4" s="15" t="str"/>
-      <x:c r="H4" s="22" t="str"/>
-      <x:c r="I4" s="15" t="str"/>
-      <x:c r="J4" s="15" t="str"/>
-      <x:c r="K4" s="15" t="str"/>
-      <x:c r="L4" s="16" t="str"/>
+      <x:c r="G4" s="15"/>
+      <x:c r="H4" s="22"/>
+      <x:c r="I4" s="15"/>
+      <x:c r="J4" s="15"/>
+      <x:c r="K4" s="15"/>
+      <x:c r="L4" s="16"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -597,6 +724,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5e16f7325b4571"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -682,127 +812,61 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>I-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="C3" s="17" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="str">
-        <x:v>10:00</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="str">
-        <x:v>11:00</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="str">
-        <x:v>Asia/Shanghai</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>抵达并前往酒店</x:v>
-      </x:c>
-      <x:c r="I3" s="23" t="str">
-        <x:v>示例交通枢纽</x:v>
-      </x:c>
-      <x:c r="J3" s="23" t="str">
-        <x:v>公共交通</x:v>
-      </x:c>
-      <x:c r="K3" s="23" t="str">
-        <x:v>B-001</x:v>
-      </x:c>
-      <x:c r="L3" s="23" t="str">
-        <x:v>Ready</x:v>
-      </x:c>
-      <x:c r="M3" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N3" s="23" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="O3" s="23" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
-      <x:c r="P3" s="24" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="12"/>
+      <x:c r="E3" s="12"/>
+      <x:c r="F3" s="12"/>
+      <x:c r="G3" s="12"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="23"/>
+      <x:c r="J3" s="23"/>
+      <x:c r="K3" s="23"/>
+      <x:c r="L3" s="23"/>
+      <x:c r="M3" s="23"/>
+      <x:c r="N3" s="23"/>
+      <x:c r="O3" s="23"/>
+      <x:c r="P3" s="24"/>
+      <x:c r="Q3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="11" t="str">
-        <x:v>I-002</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="C4" s="17" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D4" s="12" t="str">
-        <x:v>14:00</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="str">
-        <x:v>16:00</x:v>
-      </x:c>
-      <x:c r="F4" s="12" t="str">
-        <x:v>Asia/Shanghai</x:v>
-      </x:c>
-      <x:c r="G4" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="H4" s="23" t="str">
-        <x:v>城市步行</x:v>
-      </x:c>
-      <x:c r="I4" s="23" t="str">
-        <x:v>示例广场</x:v>
-      </x:c>
-      <x:c r="J4" s="23" t="str">
-        <x:v>步行</x:v>
-      </x:c>
-      <x:c r="K4" s="23" t="str"/>
-      <x:c r="L4" s="23" t="str">
-        <x:v>Planned</x:v>
-      </x:c>
-      <x:c r="M4" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N4" s="23" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="O4" s="23" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
-      <x:c r="P4" s="24" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q4" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="12"/>
+      <x:c r="C4" s="17"/>
+      <x:c r="D4" s="12"/>
+      <x:c r="E4" s="12"/>
+      <x:c r="F4" s="12"/>
+      <x:c r="G4" s="12"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="23"/>
+      <x:c r="J4" s="23"/>
+      <x:c r="K4" s="23"/>
+      <x:c r="L4" s="23"/>
+      <x:c r="M4" s="23"/>
+      <x:c r="N4" s="23"/>
+      <x:c r="O4" s="23"/>
+      <x:c r="P4" s="24"/>
+      <x:c r="Q4" s="25"/>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="14" t="str"/>
-      <x:c r="B5" s="15" t="str"/>
+      <x:c r="A5" s="14"/>
+      <x:c r="B5" s="15"/>
       <x:c r="C5" s="18"/>
-      <x:c r="D5" s="15" t="str"/>
-      <x:c r="E5" s="15" t="str"/>
-      <x:c r="F5" s="15" t="str"/>
-      <x:c r="G5" s="15" t="str"/>
-      <x:c r="H5" s="26" t="str"/>
-      <x:c r="I5" s="26" t="str"/>
-      <x:c r="J5" s="26" t="str"/>
-      <x:c r="K5" s="26" t="str"/>
-      <x:c r="L5" s="26" t="str"/>
+      <x:c r="D5" s="15"/>
+      <x:c r="E5" s="15"/>
+      <x:c r="F5" s="15"/>
+      <x:c r="G5" s="15"/>
+      <x:c r="H5" s="26"/>
+      <x:c r="I5" s="26"/>
+      <x:c r="J5" s="26"/>
+      <x:c r="K5" s="26"/>
+      <x:c r="L5" s="26"/>
       <x:c r="M5" s="26"/>
-      <x:c r="N5" s="26" t="str"/>
-      <x:c r="O5" s="26" t="str"/>
+      <x:c r="N5" s="26"/>
+      <x:c r="O5" s="26"/>
       <x:c r="P5" s="27"/>
-      <x:c r="Q5" s="28" t="str"/>
+      <x:c r="Q5" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -811,6 +875,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61fd2eb548294d19"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -884,64 +951,36 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>B-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>住宿</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>示例酒店</x:v>
-      </x:c>
-      <x:c r="D3" s="19" t="d">
-        <x:v>2030-05-01T07:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E3" s="19" t="d">
-        <x:v>2030-05-03T03:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="H3" s="12" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="I3" s="12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J3" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="K3" s="23" t="str">
-        <x:v>私人档案中的预订文件夹</x:v>
-      </x:c>
-      <x:c r="L3" s="23" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
-      <x:c r="M3" s="24" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="N3" s="25" t="str">
-        <x:v>不存放真实订单号</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="19"/>
+      <x:c r="E3" s="19"/>
+      <x:c r="F3" s="12"/>
+      <x:c r="G3" s="12"/>
+      <x:c r="H3" s="12"/>
+      <x:c r="I3" s="12"/>
+      <x:c r="J3" s="12"/>
+      <x:c r="K3" s="23"/>
+      <x:c r="L3" s="23"/>
+      <x:c r="M3" s="24"/>
+      <x:c r="N3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="15" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="15"/>
       <x:c r="D4" s="20"/>
       <x:c r="E4" s="20"/>
-      <x:c r="F4" s="15" t="str"/>
-      <x:c r="G4" s="15" t="str"/>
-      <x:c r="H4" s="15" t="str"/>
+      <x:c r="F4" s="15"/>
+      <x:c r="G4" s="15"/>
+      <x:c r="H4" s="15"/>
       <x:c r="I4" s="15"/>
-      <x:c r="J4" s="15" t="str"/>
-      <x:c r="K4" s="26" t="str"/>
-      <x:c r="L4" s="26" t="str"/>
+      <x:c r="J4" s="15"/>
+      <x:c r="K4" s="26"/>
+      <x:c r="L4" s="26"/>
       <x:c r="M4" s="27"/>
-      <x:c r="N4" s="28" t="str"/>
+      <x:c r="N4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -950,6 +989,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac518cad28734e68"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1003,42 +1045,26 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>T-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>确认</x:v>
-      </x:c>
-      <x:c r="C3" s="23" t="str">
-        <x:v>出发前复核住宿</x:v>
-      </x:c>
-      <x:c r="D3" s="23" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="E3" s="29" t="d">
-        <x:v>2030-04-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str"/>
-      <x:c r="H3" s="23" t="str">
-        <x:v>B-001</x:v>
-      </x:c>
-      <x:c r="I3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="23"/>
+      <x:c r="D3" s="23"/>
+      <x:c r="E3" s="29"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="26" t="str"/>
-      <x:c r="D4" s="26" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="26"/>
+      <x:c r="D4" s="26"/>
       <x:c r="E4" s="30"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="26" t="str"/>
-      <x:c r="H4" s="26" t="str"/>
-      <x:c r="I4" s="28" t="str"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="26"/>
+      <x:c r="H4" s="26"/>
+      <x:c r="I4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1047,6 +1073,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra98688a8d8664625"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1108,52 +1137,30 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>P-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>本次旅行</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>节奏</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="str">
-        <x:v>硬约束</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="str">
-        <x:v>所有人</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>每日步行不超过虚构上限</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str">
-        <x:v>用户明确说明</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="I3" s="29" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="J3" s="29" t="d">
-        <x:v>2030-05-03T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="K3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="12"/>
+      <x:c r="E3" s="12"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="29"/>
+      <x:c r="J3" s="29"/>
+      <x:c r="K3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="15" t="str"/>
-      <x:c r="D4" s="15" t="str"/>
-      <x:c r="E4" s="15" t="str"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="26" t="str"/>
-      <x:c r="H4" s="26" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="15"/>
+      <x:c r="D4" s="15"/>
+      <x:c r="E4" s="15"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="26"/>
+      <x:c r="H4" s="26"/>
       <x:c r="I4" s="30"/>
       <x:c r="J4" s="30"/>
-      <x:c r="K4" s="28" t="str"/>
+      <x:c r="K4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -1165,6 +1172,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc39f38c7055641f0"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1210,35 +1220,28 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="B3" s="19" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="D3" s="23" t="str">
-        <x:v>建立初始版本</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:v>创建虚构示例行程</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str"/>
-      <x:c r="G3" s="25" t="str"/>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="19"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="23"/>
+      <x:c r="E3" s="23"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
+      <x:c r="A4" s="14"/>
       <x:c r="B4" s="20"/>
-      <x:c r="C4" s="15" t="str"/>
-      <x:c r="D4" s="26" t="str"/>
-      <x:c r="E4" s="26" t="str"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="28" t="str"/>
+      <x:c r="C4" s="15"/>
+      <x:c r="D4" s="26"/>
+      <x:c r="E4" s="26"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R142c83512b46467e"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1284,57 +1287,31 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>旅行负责人</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="D3" s="23" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str"/>
-      <x:c r="F3" s="23" t="str">
-        <x:v>最终确认</x:v>
-      </x:c>
-      <x:c r="G3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="23"/>
+      <x:c r="E3" s="23"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="11" t="str">
-        <x:v>M-002</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>同行者 A</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
-        <x:v>Member</x:v>
-      </x:c>
-      <x:c r="D4" s="23" t="str">
-        <x:v>同行者</x:v>
-      </x:c>
-      <x:c r="E4" s="23" t="str">
-        <x:v>避免太晚返程</x:v>
-      </x:c>
-      <x:c r="F4" s="23" t="str">
-        <x:v>提出意见</x:v>
-      </x:c>
-      <x:c r="G4" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="12"/>
+      <x:c r="C4" s="12"/>
+      <x:c r="D4" s="23"/>
+      <x:c r="E4" s="23"/>
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="25"/>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="14" t="str"/>
-      <x:c r="B5" s="15" t="str"/>
-      <x:c r="C5" s="15" t="str"/>
-      <x:c r="D5" s="26" t="str"/>
-      <x:c r="E5" s="26" t="str"/>
-      <x:c r="F5" s="26" t="str"/>
-      <x:c r="G5" s="28" t="str"/>
+      <x:c r="A5" s="14"/>
+      <x:c r="B5" s="15"/>
+      <x:c r="C5" s="15"/>
+      <x:c r="D5" s="26"/>
+      <x:c r="E5" s="26"/>
+      <x:c r="F5" s="26"/>
+      <x:c r="G5" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1343,6 +1320,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R159238e89c2a49cd"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1400,44 +1380,28 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>PR-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>M-002</x:v>
-      </x:c>
-      <x:c r="C3" s="17" t="d">
-        <x:v>2030-04-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="str">
-        <x:v>2030-05-02</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:v>晚餐提前一小时</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>避免太晚返程</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="I3" s="23" t="str"/>
-      <x:c r="J3" s="25" t="str"/>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="12"/>
+      <x:c r="E3" s="23"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="23"/>
+      <x:c r="J3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
       <x:c r="C4" s="18"/>
-      <x:c r="D4" s="15" t="str"/>
-      <x:c r="E4" s="26" t="str"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="26" t="str"/>
-      <x:c r="H4" s="26" t="str"/>
-      <x:c r="I4" s="26" t="str"/>
-      <x:c r="J4" s="28" t="str"/>
+      <x:c r="D4" s="15"/>
+      <x:c r="E4" s="26"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="26"/>
+      <x:c r="H4" s="26"/>
+      <x:c r="I4" s="26"/>
+      <x:c r="J4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1446,5 +1410,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cbcef37f26a4c73"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: separate blank template from example archive (#5)
</commit_message>
<xml_diff>
--- a/skill/travel-os/assets/TravelOS-Template.xlsx
+++ b/skill/travel-os/assets/TravelOS-Template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travel Overview" sheetId="1" r:id="R1923f46351a44bca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Plan" sheetId="2" r:id="R57f2af995ad545fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="3" r:id="R3f382a0ca7ce463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="4" r:id="Re882fef17dff4f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferences" sheetId="5" r:id="R10c94c6a9c9a44f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="6" r:id="R0d82132e5d19404c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" r:id="R5b4c9e3a47264ad5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposals" sheetId="8" r:id="R0f4a7277c3624dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travel Overview" sheetId="1" r:id="Rb064bddc82b44833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Plan" sheetId="2" r:id="R90206dae9334462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="3" r:id="Rc155e68ab1c24824"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="4" r:id="R598f5d44f3ad4f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferences" sheetId="5" r:id="R4681bcd0bed946a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="6" r:id="Rdba29f382d9d4841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" r:id="Rc3b476cd2b3e4bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposals" sheetId="8" r:id="R974b8a2f51674eca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -281,6 +281,157 @@
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TravelOverview" displayName="TravelOverview" ref="A2:L4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="Trip ID"/>
+    <x:tableColumn id="2" name="旅行标题"/>
+    <x:tableColumn id="3" name="目的地"/>
+    <x:tableColumn id="4" name="开始日期"/>
+    <x:tableColumn id="5" name="结束日期"/>
+    <x:tableColumn id="6" name="人数"/>
+    <x:tableColumn id="7" name="负责人"/>
+    <x:tableColumn id="8" name="Active Version"/>
+    <x:tableColumn id="9" name="旅行阶段"/>
+    <x:tableColumn id="10" name="状态"/>
+    <x:tableColumn id="11" name="主时区"/>
+    <x:tableColumn id="12" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DailyPlan" displayName="DailyPlan" ref="A2:Q5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="17">
+    <x:tableColumn id="1" name="项目ID"/>
+    <x:tableColumn id="2" name="版本"/>
+    <x:tableColumn id="3" name="日期"/>
+    <x:tableColumn id="4" name="开始"/>
+    <x:tableColumn id="5" name="结束"/>
+    <x:tableColumn id="6" name="时区"/>
+    <x:tableColumn id="7" name="城市"/>
+    <x:tableColumn id="8" name="活动"/>
+    <x:tableColumn id="9" name="地点"/>
+    <x:tableColumn id="10" name="交通"/>
+    <x:tableColumn id="11" name="预订ID"/>
+    <x:tableColumn id="12" name="执行状态"/>
+    <x:tableColumn id="13" name="费用"/>
+    <x:tableColumn id="14" name="币种"/>
+    <x:tableColumn id="15" name="来源"/>
+    <x:tableColumn id="16" name="核验时间"/>
+    <x:tableColumn id="17" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Bookings" displayName="Bookings" ref="A2:N4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="14">
+    <x:tableColumn id="1" name="预订ID"/>
+    <x:tableColumn id="2" name="类别"/>
+    <x:tableColumn id="3" name="供应方"/>
+    <x:tableColumn id="4" name="开始时间"/>
+    <x:tableColumn id="5" name="结束时间"/>
+    <x:tableColumn id="6" name="城市"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="可退"/>
+    <x:tableColumn id="9" name="金额"/>
+    <x:tableColumn id="10" name="币种"/>
+    <x:tableColumn id="11" name="凭证位置"/>
+    <x:tableColumn id="12" name="来源"/>
+    <x:tableColumn id="13" name="核验时间"/>
+    <x:tableColumn id="14" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Checklist" displayName="Checklist" ref="A2:I4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务ID"/>
+    <x:tableColumn id="2" name="类别"/>
+    <x:tableColumn id="3" name="任务"/>
+    <x:tableColumn id="4" name="负责人"/>
+    <x:tableColumn id="5" name="截止日期"/>
+    <x:tableColumn id="6" name="状态"/>
+    <x:tableColumn id="7" name="依赖"/>
+    <x:tableColumn id="8" name="关联ID"/>
+    <x:tableColumn id="9" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Preferences" displayName="Preferences" ref="A2:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="偏好ID"/>
+    <x:tableColumn id="2" name="范围"/>
+    <x:tableColumn id="3" name="类别"/>
+    <x:tableColumn id="4" name="优先级"/>
+    <x:tableColumn id="5" name="适用人"/>
+    <x:tableColumn id="6" name="偏好或约束"/>
+    <x:tableColumn id="7" name="证据"/>
+    <x:tableColumn id="8" name="置信度"/>
+    <x:tableColumn id="9" name="生效日期"/>
+    <x:tableColumn id="10" name="失效日期"/>
+    <x:tableColumn id="11" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ChangeLog" displayName="ChangeLog" ref="A2:G4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="版本"/>
+    <x:tableColumn id="2" name="创建时间"/>
+    <x:tableColumn id="3" name="作者"/>
+    <x:tableColumn id="4" name="原因"/>
+    <x:tableColumn id="5" name="变更摘要"/>
+    <x:tableColumn id="6" name="上一版本"/>
+    <x:tableColumn id="7" name="档案哈希"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Members" displayName="Members" ref="A2:G5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="成员ID"/>
+    <x:tableColumn id="2" name="显示名"/>
+    <x:tableColumn id="3" name="角色"/>
+    <x:tableColumn id="4" name="同行关系"/>
+    <x:tableColumn id="5" name="本次需求"/>
+    <x:tableColumn id="6" name="权限"/>
+    <x:tableColumn id="7" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Proposals" displayName="Proposals" ref="A2:J4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="提案ID"/>
+    <x:tableColumn id="2" name="提交人"/>
+    <x:tableColumn id="3" name="日期"/>
+    <x:tableColumn id="4" name="影响项目或日期"/>
+    <x:tableColumn id="5" name="提案"/>
+    <x:tableColumn id="6" name="原因"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="决策人"/>
+    <x:tableColumn id="9" name="处理结果"/>
+    <x:tableColumn id="10" name="结果版本"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -536,56 +687,32 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>DEMO-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>示例城市周末</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="D3" s="17" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E3" s="17" t="d">
-        <x:v>2030-05-03T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="H3" s="21" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="I3" s="12" t="str">
-        <x:v>行前规划</x:v>
-      </x:c>
-      <x:c r="J3" s="12" t="str">
-        <x:v>Active</x:v>
-      </x:c>
-      <x:c r="K3" s="12" t="str">
-        <x:v>Asia/Shanghai</x:v>
-      </x:c>
-      <x:c r="L3" s="13" t="str">
-        <x:v>本行仅为虚构示例，请替换</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="12"/>
+      <x:c r="G3" s="12"/>
+      <x:c r="H3" s="21"/>
+      <x:c r="I3" s="12"/>
+      <x:c r="J3" s="12"/>
+      <x:c r="K3" s="12"/>
+      <x:c r="L3" s="13"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="15" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="15"/>
       <x:c r="D4" s="18"/>
       <x:c r="E4" s="18"/>
       <x:c r="F4" s="15"/>
-      <x:c r="G4" s="15" t="str"/>
-      <x:c r="H4" s="22" t="str"/>
-      <x:c r="I4" s="15" t="str"/>
-      <x:c r="J4" s="15" t="str"/>
-      <x:c r="K4" s="15" t="str"/>
-      <x:c r="L4" s="16" t="str"/>
+      <x:c r="G4" s="15"/>
+      <x:c r="H4" s="22"/>
+      <x:c r="I4" s="15"/>
+      <x:c r="J4" s="15"/>
+      <x:c r="K4" s="15"/>
+      <x:c r="L4" s="16"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -597,6 +724,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5e16f7325b4571"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -682,127 +812,61 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>I-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="C3" s="17" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="str">
-        <x:v>10:00</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="str">
-        <x:v>11:00</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="str">
-        <x:v>Asia/Shanghai</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>抵达并前往酒店</x:v>
-      </x:c>
-      <x:c r="I3" s="23" t="str">
-        <x:v>示例交通枢纽</x:v>
-      </x:c>
-      <x:c r="J3" s="23" t="str">
-        <x:v>公共交通</x:v>
-      </x:c>
-      <x:c r="K3" s="23" t="str">
-        <x:v>B-001</x:v>
-      </x:c>
-      <x:c r="L3" s="23" t="str">
-        <x:v>Ready</x:v>
-      </x:c>
-      <x:c r="M3" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N3" s="23" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="O3" s="23" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
-      <x:c r="P3" s="24" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="12"/>
+      <x:c r="E3" s="12"/>
+      <x:c r="F3" s="12"/>
+      <x:c r="G3" s="12"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="23"/>
+      <x:c r="J3" s="23"/>
+      <x:c r="K3" s="23"/>
+      <x:c r="L3" s="23"/>
+      <x:c r="M3" s="23"/>
+      <x:c r="N3" s="23"/>
+      <x:c r="O3" s="23"/>
+      <x:c r="P3" s="24"/>
+      <x:c r="Q3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="11" t="str">
-        <x:v>I-002</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="C4" s="17" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D4" s="12" t="str">
-        <x:v>14:00</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="str">
-        <x:v>16:00</x:v>
-      </x:c>
-      <x:c r="F4" s="12" t="str">
-        <x:v>Asia/Shanghai</x:v>
-      </x:c>
-      <x:c r="G4" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="H4" s="23" t="str">
-        <x:v>城市步行</x:v>
-      </x:c>
-      <x:c r="I4" s="23" t="str">
-        <x:v>示例广场</x:v>
-      </x:c>
-      <x:c r="J4" s="23" t="str">
-        <x:v>步行</x:v>
-      </x:c>
-      <x:c r="K4" s="23" t="str"/>
-      <x:c r="L4" s="23" t="str">
-        <x:v>Planned</x:v>
-      </x:c>
-      <x:c r="M4" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N4" s="23" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="O4" s="23" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
-      <x:c r="P4" s="24" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q4" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="12"/>
+      <x:c r="C4" s="17"/>
+      <x:c r="D4" s="12"/>
+      <x:c r="E4" s="12"/>
+      <x:c r="F4" s="12"/>
+      <x:c r="G4" s="12"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="23"/>
+      <x:c r="J4" s="23"/>
+      <x:c r="K4" s="23"/>
+      <x:c r="L4" s="23"/>
+      <x:c r="M4" s="23"/>
+      <x:c r="N4" s="23"/>
+      <x:c r="O4" s="23"/>
+      <x:c r="P4" s="24"/>
+      <x:c r="Q4" s="25"/>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="14" t="str"/>
-      <x:c r="B5" s="15" t="str"/>
+      <x:c r="A5" s="14"/>
+      <x:c r="B5" s="15"/>
       <x:c r="C5" s="18"/>
-      <x:c r="D5" s="15" t="str"/>
-      <x:c r="E5" s="15" t="str"/>
-      <x:c r="F5" s="15" t="str"/>
-      <x:c r="G5" s="15" t="str"/>
-      <x:c r="H5" s="26" t="str"/>
-      <x:c r="I5" s="26" t="str"/>
-      <x:c r="J5" s="26" t="str"/>
-      <x:c r="K5" s="26" t="str"/>
-      <x:c r="L5" s="26" t="str"/>
+      <x:c r="D5" s="15"/>
+      <x:c r="E5" s="15"/>
+      <x:c r="F5" s="15"/>
+      <x:c r="G5" s="15"/>
+      <x:c r="H5" s="26"/>
+      <x:c r="I5" s="26"/>
+      <x:c r="J5" s="26"/>
+      <x:c r="K5" s="26"/>
+      <x:c r="L5" s="26"/>
       <x:c r="M5" s="26"/>
-      <x:c r="N5" s="26" t="str"/>
-      <x:c r="O5" s="26" t="str"/>
+      <x:c r="N5" s="26"/>
+      <x:c r="O5" s="26"/>
       <x:c r="P5" s="27"/>
-      <x:c r="Q5" s="28" t="str"/>
+      <x:c r="Q5" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -811,6 +875,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61fd2eb548294d19"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -884,64 +951,36 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>B-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>住宿</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>示例酒店</x:v>
-      </x:c>
-      <x:c r="D3" s="19" t="d">
-        <x:v>2030-05-01T07:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E3" s="19" t="d">
-        <x:v>2030-05-03T03:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="str">
-        <x:v>示例城</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="str">
-        <x:v>已确认</x:v>
-      </x:c>
-      <x:c r="H3" s="12" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="I3" s="12" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J3" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="K3" s="23" t="str">
-        <x:v>私人档案中的预订文件夹</x:v>
-      </x:c>
-      <x:c r="L3" s="23" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
-      <x:c r="M3" s="24" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="N3" s="25" t="str">
-        <x:v>不存放真实订单号</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="19"/>
+      <x:c r="E3" s="19"/>
+      <x:c r="F3" s="12"/>
+      <x:c r="G3" s="12"/>
+      <x:c r="H3" s="12"/>
+      <x:c r="I3" s="12"/>
+      <x:c r="J3" s="12"/>
+      <x:c r="K3" s="23"/>
+      <x:c r="L3" s="23"/>
+      <x:c r="M3" s="24"/>
+      <x:c r="N3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="15" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="15"/>
       <x:c r="D4" s="20"/>
       <x:c r="E4" s="20"/>
-      <x:c r="F4" s="15" t="str"/>
-      <x:c r="G4" s="15" t="str"/>
-      <x:c r="H4" s="15" t="str"/>
+      <x:c r="F4" s="15"/>
+      <x:c r="G4" s="15"/>
+      <x:c r="H4" s="15"/>
       <x:c r="I4" s="15"/>
-      <x:c r="J4" s="15" t="str"/>
-      <x:c r="K4" s="26" t="str"/>
-      <x:c r="L4" s="26" t="str"/>
+      <x:c r="J4" s="15"/>
+      <x:c r="K4" s="26"/>
+      <x:c r="L4" s="26"/>
       <x:c r="M4" s="27"/>
-      <x:c r="N4" s="28" t="str"/>
+      <x:c r="N4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -950,6 +989,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac518cad28734e68"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1003,42 +1045,26 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>T-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>确认</x:v>
-      </x:c>
-      <x:c r="C3" s="23" t="str">
-        <x:v>出发前复核住宿</x:v>
-      </x:c>
-      <x:c r="D3" s="23" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="E3" s="29" t="d">
-        <x:v>2030-04-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str"/>
-      <x:c r="H3" s="23" t="str">
-        <x:v>B-001</x:v>
-      </x:c>
-      <x:c r="I3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="23"/>
+      <x:c r="D3" s="23"/>
+      <x:c r="E3" s="29"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="26" t="str"/>
-      <x:c r="D4" s="26" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="26"/>
+      <x:c r="D4" s="26"/>
       <x:c r="E4" s="30"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="26" t="str"/>
-      <x:c r="H4" s="26" t="str"/>
-      <x:c r="I4" s="28" t="str"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="26"/>
+      <x:c r="H4" s="26"/>
+      <x:c r="I4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1047,6 +1073,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra98688a8d8664625"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1108,52 +1137,30 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>P-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>本次旅行</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>节奏</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="str">
-        <x:v>硬约束</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="str">
-        <x:v>所有人</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>每日步行不超过虚构上限</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str">
-        <x:v>用户明确说明</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="I3" s="29" t="d">
-        <x:v>2030-05-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="J3" s="29" t="d">
-        <x:v>2030-05-03T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="K3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="12"/>
+      <x:c r="E3" s="12"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="29"/>
+      <x:c r="J3" s="29"/>
+      <x:c r="K3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="15" t="str"/>
-      <x:c r="D4" s="15" t="str"/>
-      <x:c r="E4" s="15" t="str"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="26" t="str"/>
-      <x:c r="H4" s="26" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="15"/>
+      <x:c r="D4" s="15"/>
+      <x:c r="E4" s="15"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="26"/>
+      <x:c r="H4" s="26"/>
       <x:c r="I4" s="30"/>
       <x:c r="J4" s="30"/>
-      <x:c r="K4" s="28" t="str"/>
+      <x:c r="K4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -1165,6 +1172,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc39f38c7055641f0"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1210,35 +1220,28 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>v0.1.0</x:v>
-      </x:c>
-      <x:c r="B3" s="19" t="d">
-        <x:v>2030-04-01T02:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="D3" s="23" t="str">
-        <x:v>建立初始版本</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:v>创建虚构示例行程</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str"/>
-      <x:c r="G3" s="25" t="str"/>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="19"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="23"/>
+      <x:c r="E3" s="23"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
+      <x:c r="A4" s="14"/>
       <x:c r="B4" s="20"/>
-      <x:c r="C4" s="15" t="str"/>
-      <x:c r="D4" s="26" t="str"/>
-      <x:c r="E4" s="26" t="str"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="28" t="str"/>
+      <x:c r="C4" s="15"/>
+      <x:c r="D4" s="26"/>
+      <x:c r="E4" s="26"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R142c83512b46467e"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1284,57 +1287,31 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>旅行负责人</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="D3" s="23" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str"/>
-      <x:c r="F3" s="23" t="str">
-        <x:v>最终确认</x:v>
-      </x:c>
-      <x:c r="G3" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="23"/>
+      <x:c r="E3" s="23"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="11" t="str">
-        <x:v>M-002</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>同行者 A</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
-        <x:v>Member</x:v>
-      </x:c>
-      <x:c r="D4" s="23" t="str">
-        <x:v>同行者</x:v>
-      </x:c>
-      <x:c r="E4" s="23" t="str">
-        <x:v>避免太晚返程</x:v>
-      </x:c>
-      <x:c r="F4" s="23" t="str">
-        <x:v>提出意见</x:v>
-      </x:c>
-      <x:c r="G4" s="25" t="str">
-        <x:v>虚构示例</x:v>
-      </x:c>
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="12"/>
+      <x:c r="C4" s="12"/>
+      <x:c r="D4" s="23"/>
+      <x:c r="E4" s="23"/>
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="25"/>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="14" t="str"/>
-      <x:c r="B5" s="15" t="str"/>
-      <x:c r="C5" s="15" t="str"/>
-      <x:c r="D5" s="26" t="str"/>
-      <x:c r="E5" s="26" t="str"/>
-      <x:c r="F5" s="26" t="str"/>
-      <x:c r="G5" s="28" t="str"/>
+      <x:c r="A5" s="14"/>
+      <x:c r="B5" s="15"/>
+      <x:c r="C5" s="15"/>
+      <x:c r="D5" s="26"/>
+      <x:c r="E5" s="26"/>
+      <x:c r="F5" s="26"/>
+      <x:c r="G5" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1343,6 +1320,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R159238e89c2a49cd"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1400,44 +1380,28 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>PR-001</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>M-002</x:v>
-      </x:c>
-      <x:c r="C3" s="17" t="d">
-        <x:v>2030-04-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="str">
-        <x:v>2030-05-02</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:v>晚餐提前一小时</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>避免太晚返程</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="I3" s="23" t="str"/>
-      <x:c r="J3" s="25" t="str"/>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="12"/>
+      <x:c r="E3" s="23"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="23"/>
+      <x:c r="J3" s="25"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="14" t="str"/>
-      <x:c r="B4" s="15" t="str"/>
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="15"/>
       <x:c r="C4" s="18"/>
-      <x:c r="D4" s="15" t="str"/>
-      <x:c r="E4" s="26" t="str"/>
-      <x:c r="F4" s="26" t="str"/>
-      <x:c r="G4" s="26" t="str"/>
-      <x:c r="H4" s="26" t="str"/>
-      <x:c r="I4" s="26" t="str"/>
-      <x:c r="J4" s="28" t="str"/>
+      <x:c r="D4" s="15"/>
+      <x:c r="E4" s="26"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="26"/>
+      <x:c r="H4" s="26"/>
+      <x:c r="I4" s="26"/>
+      <x:c r="J4" s="28"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1446,5 +1410,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cbcef37f26a4c73"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>